<commit_message>
feat: hoàn thành Bài 02 (JR-02) boxing, Integer cache
</commit_message>
<xml_diff>
--- a/tracker/bai-tap-java.xlsx
+++ b/tracker/bai-tap-java.xlsx
@@ -629,7 +629,12 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đã làm</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat: hoàn thành Bài 03 (JR-03) String và StringBuilder
</commit_message>
<xml_diff>
--- a/tracker/bai-tap-java.xlsx
+++ b/tracker/bai-tap-java.xlsx
@@ -693,7 +693,12 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đã làm</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>

</xml_diff>